<commit_message>
Fix formula; replace checkboxes with click-to-select county names
Formula fix: replaced SORT(FILTER(…), {1,3}, {TRUE,TRUE}) — Excel array
syntax Google Sheets rejects — with a QUERY whose WHERE clause is built
dynamically using LET + TEXTJOIN:
  county_part  → "A MATCHES 'Adams|Allen|…' AND "  (blank = all counties)
  type_part    → "C = 'House' AND "                (blank = all types)
  num_part     → "D = 47 AND "                     (blank = all numbers)
Trailing ' AND ' stripped with LEFT(); ORDER BY handles sorting natively.

Click-to-select UX: county name cells (cols B and D, rows 6-51) now toggle
selection when clicked via onSelectionChange in Apps Script. Hidden state
columns (C and E, width 3) store TRUE/FALSE. Conditional formatting lights
the county name gold when its state cell is TRUE — no separate tab needed.

https://claude.ai/code/session_01BLbS7KUkKuAXVcodzTcFdz
</commit_message>
<xml_diff>
--- a/Indiana_County_Candidates_2026.xlsx
+++ b/Indiana_County_Candidates_2026.xlsx
@@ -51,14 +51,11 @@
       <sz val="11"/>
     </font>
     <font>
+      <b val="1"/>
       <color rgb="000C2340"/>
       <sz val="10"/>
     </font>
     <font>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
       <color rgb="000C2340"/>
       <sz val="10"/>
     </font>
@@ -86,6 +83,9 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
@@ -187,20 +187,20 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -208,7 +208,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -217,25 +217,25 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -246,7 +246,19 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="000C2340"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F5DFA0"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="1"/>
@@ -654,14 +666,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M52"/>
+  <dimension ref="A1:M60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="1" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="3" customWidth="1" min="5" max="5"/>
     <col width="2" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
@@ -683,7 +695,7 @@
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Check counties on the left to filter results on the right.  Leave all unchecked to show every county.  Use the District Type and # fields to narrow by district.</t>
+          <t>Click a county name to select or deselect it — selected counties highlight gold.  Leave all unselected to show every county.  Use the Type and Dist # fields to filter by district.</t>
         </is>
       </c>
       <c r="F2" s="2" t="n"/>
@@ -698,7 +710,7 @@
         </is>
       </c>
       <c r="C4" s="5">
-        <f>LET(n,COUNTIF(C6:C51,TRUE)+COUNTIF(E6:E51,TRUE),IF(n=0,"All 92 counties",n&amp;" of 92 selected"))</f>
+        <f>LET(n,COUNTIF(C6:C51,TRUE)+COUNTIF(E6:E51,TRUE),IF(n=0,"All 92 counties — click to filter",n&amp;" of 92 selected"))</f>
         <v/>
       </c>
       <c r="F4" s="2" t="n"/>
@@ -729,21 +741,13 @@
           <t>County</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="C5" s="7" t="inlineStr"/>
       <c r="D5" s="7" t="inlineStr">
         <is>
           <t>County</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="E5" s="7" t="inlineStr"/>
       <c r="F5" s="2" t="n"/>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -800,7 +804,7 @@
       </c>
       <c r="F6" s="2" t="n"/>
       <c r="G6">
-        <f>IFERROR(LET(checked,COUNTIF(C6:C51,TRUE)+COUNTIF(E6:E51,TRUE),county_match,IF(checked=0,TRUE,COUNTIF(FILTER({B6:B51;D6:D51},{C6:C51;E6:E51}),'All Data'!A2:A737)&gt;0),type_match,(I4="All Types")+('All Data'!C2:C737=I4)&gt;0,num_match,(LEN(TRIM(L4))=0)+('All Data'!D2:D737=IFERROR(VALUE(L4),0))&gt;0,SORT(FILTER({'All Data'!E2:E737,'All Data'!C2:C737,'All Data'!D2:D737,'All Data'!F2:F737,'All Data'!G2:G737,'All Data'!H2:H737,'All Data'!J2:J737},county_match*type_match*num_match),{{1,3}},{{TRUE,TRUE}})),"No candidates match the selected filters.")</f>
+        <f>IFERROR(LET(n,COUNTIF(C6:C51,TRUE)+COUNTIF(E6:E51,TRUE),county_part,IF(n=0,"","A MATCHES '"&amp;TEXTJOIN("|",TRUE,IF(C6:C51,B6:B51,""),IF(E6:E51,D6:D51,""))&amp;"' AND "),type_part,IF(I4="All Types","","C = '"&amp;I4&amp;"' AND "),num_part,IF(LEN(TRIM(L4))=0,"","D = "&amp;IFERROR(VALUE(L4),0)&amp;" AND "),all_parts,county_part&amp;type_part&amp;num_part,where_str,IF(LEN(all_parts)=0,"","WHERE "&amp;LEFT(all_parts,LEN(all_parts)-5)),QUERY('All Data'!A:J,"SELECT E,C,D,F,G,H,J "&amp;where_str&amp;" ORDER BY B ASC,D ASC,I ASC",1)),"No candidates match the selected filters.")</f>
         <v/>
       </c>
     </row>
@@ -1661,6 +1665,30 @@
     </row>
     <row r="52">
       <c r="F52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="F53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="F54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="F55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="F56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="F57" s="2" t="n"/>
+    </row>
+    <row r="58">
+      <c r="F58" s="2" t="n"/>
+    </row>
+    <row r="59">
+      <c r="F59" s="2" t="n"/>
+    </row>
+    <row r="60">
+      <c r="F60" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1668,19 +1696,29 @@
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A1:M1"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6:B51">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$C6=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D6:D51">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>$E6=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="K6:K5000">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="3" dxfId="1">
       <formula>$K6="D"</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
+    <cfRule type="expression" priority="4" dxfId="2">
       <formula>$K6="R"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="2">
+    <cfRule type="expression" priority="5" dxfId="3">
       <formula>AND($K6&lt;&gt;"D",$K6&lt;&gt;"R",$K6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L6:L5000">
-    <cfRule type="expression" priority="4" dxfId="3">
+    <cfRule type="expression" priority="6" dxfId="4">
       <formula>LEFT($L6,3)="Won"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -62211,7 +62249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -62227,35 +62265,35 @@
     <row r="3">
       <c r="A3" s="21" t="inlineStr">
         <is>
-          <t>WHAT THIS SCRIPT ADDS:</t>
+          <t>WHAT THIS SCRIPT DOES:</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="22" t="inlineStr">
         <is>
-          <t>• IRS Tools menu → Select All / Clear All counties with one click</t>
+          <t>• onSelectionChange — clicking a county name toggles it selected/unselected</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="22" t="inlineStr">
         <is>
-          <t>• Toast notification when filters or checkboxes change</t>
+          <t>• onEdit — toast notification when filters change</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="22" t="inlineStr">
         <is>
-          <t>• Reset District Filter menu item</t>
+          <t>• IRS Tools menu — Select All / Clear All / Reset District Filter</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>HOW TO ADD:</t>
+          <t>HOW TO INSTALL (one-time setup):</t>
         </is>
       </c>
     </row>
@@ -62269,35 +62307,28 @@
     <row r="10">
       <c r="A10" s="22" t="inlineStr">
         <is>
-          <t>2. Delete placeholder code, paste everything from row 17 onward</t>
+          <t>2. Delete any placeholder code, paste ALL code from row 17 onward</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="22" t="inlineStr">
         <is>
-          <t>3. Save (Ctrl+S), close Apps Script tab, reload spreadsheet</t>
+          <t>3. Save (Ctrl+S / Cmd+S), then close the Apps Script tab</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="22" t="inlineStr">
         <is>
-          <t>4. IRS Tools menu appears — run Select All or Clear All to bulk-toggle</t>
+          <t>4. Reload the spreadsheet — IRS Tools menu appears in the menu bar</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="22" t="inlineStr">
         <is>
-          <t>5. IMPORTANT: also select cells C6:C51 and E6:E51 on the Lookup tab,</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   then Format → Checkbox to turn them into real toggle checkboxes</t>
+          <t>5. onSelectionChange activates immediately; clicking county names now toggles them</t>
         </is>
       </c>
     </row>
@@ -62335,484 +62366,611 @@
     <row r="21">
       <c r="A21" s="24" t="inlineStr">
         <is>
-          <t>function onOpen() {</t>
+          <t>// ---- Custom menu ----</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SpreadsheetApp.getUi()</t>
+          <t>function onOpen() {</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    .createMenu('IRS Tools')</t>
+          <t xml:space="preserve">  SpreadsheetApp.getUi()</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    .addItem('Select All Counties',   'selectAllCounties')</t>
+          <t xml:space="preserve">    .createMenu('IRS Tools')</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    .addItem('Clear All Counties',    'clearAllCounties')</t>
+          <t xml:space="preserve">    .addItem('Select All Counties',   'selectAllCounties')</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    .addSeparator()</t>
+          <t xml:space="preserve">    .addItem('Clear All Counties',    'clearAllCounties')</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    .addItem('Reset District Filter', 'resetDistrictFilter')</t>
+          <t xml:space="preserve">    .addSeparator()</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    .addSeparator()</t>
+          <t xml:space="preserve">    .addItem('Reset District Filter', 'resetDistrictFilter')</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    .addItem('Go to By District tab', 'goToByDistrict')</t>
+          <t xml:space="preserve">    .addSeparator()</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    .addToUi();</t>
+          <t xml:space="preserve">    .addItem('Go to By District tab', 'goToByDistrict')</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="24" t="inlineStr">
         <is>
+          <t xml:space="preserve">    .addToUi();</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="24" t="inlineStr">
+        <is>
           <t>}</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="24" t="inlineStr"/>
-    </row>
     <row r="33">
-      <c r="A33" s="24" t="inlineStr">
-        <is>
-          <t>// ---- County helpers ----</t>
-        </is>
-      </c>
+      <c r="A33" s="24" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>function selectAllCounties() {</t>
+          <t>// ---- Click a county name to toggle selection ----</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  const lu = SpreadsheetApp.getActiveSpreadsheet().getSheetByName('Lookup');</t>
+          <t>// County name cells: col B (2) rows 6-51 → state in col C (3)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  lu.getRange('C6:C51').setValue(true);</t>
+          <t>//                   col D (4) rows 6-51 → state in col E (5)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  lu.getRange('E6:E51').setValue(true);</t>
+          <t>function onSelectionChange(e) {</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SpreadsheetApp.getActiveSpreadsheet()</t>
+          <t xml:space="preserve">  const sheet = e.range.getSheet();</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    .toast('All 92 counties selected.', 'IRS Tools', 3);</t>
+          <t xml:space="preserve">  if (sheet.getName() !== 'Lookup') return;</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="24" t="inlineStr">
-        <is>
-          <t>}</t>
-        </is>
-      </c>
+      <c r="A40" s="24" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="24" t="inlineStr"/>
+      <c r="A41" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  // Only act on single-cell clicks (ignore drag selections)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="24" t="inlineStr">
         <is>
-          <t>function clearAllCounties() {</t>
+          <t xml:space="preserve">  if (e.range.getNumRows() !== 1 || e.range.getNumColumns() !== 1) return;</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  const lu = SpreadsheetApp.getActiveSpreadsheet().getSheetByName('Lookup');</t>
-        </is>
-      </c>
+      <c r="A43" s="24" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  lu.getRange('C6:C51').setValue(false);</t>
+          <t xml:space="preserve">  const col = e.range.getColumn();</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  lu.getRange('E6:E51').setValue(false);</t>
+          <t xml:space="preserve">  const row = e.range.getRow();</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SpreadsheetApp.getActiveSpreadsheet()</t>
+          <t xml:space="preserve">  if (row &lt; 6 || row &gt; 51) return;</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    .toast('Cleared — showing all 92 counties.', 'IRS Tools', 3);</t>
-        </is>
-      </c>
+      <c r="A47" s="24" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="24" t="inlineStr">
         <is>
-          <t>}</t>
+          <t xml:space="preserve">  let stateCol = null;</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="24" t="inlineStr"/>
+      <c r="A49" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  if (col === 2) stateCol = 3;   // clicked left county name → toggle col C</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="24" t="inlineStr">
         <is>
-          <t>// ---- District filter reset ----</t>
+          <t xml:space="preserve">  if (col === 4) stateCol = 5;   // clicked right county name → toggle col E</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="24" t="inlineStr">
         <is>
-          <t>function resetDistrictFilter() {</t>
+          <t xml:space="preserve">  if (!stateCol) return;</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  const lu = SpreadsheetApp.getActiveSpreadsheet().getSheetByName('Lookup');</t>
-        </is>
-      </c>
+      <c r="A52" s="24" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  lu.getRange('I4').setValue('All Types');</t>
+          <t xml:space="preserve">  const stateCell = sheet.getRange(row, stateCol);</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  lu.getRange('L4').clearContent();</t>
+          <t xml:space="preserve">  stateCell.setValue(!stateCell.getValue());</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SpreadsheetApp.getActiveSpreadsheet()</t>
+          <t>}</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    .toast('District filter reset.', 'IRS Tools', 2);</t>
-        </is>
-      </c>
+      <c r="A56" s="24" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="24" t="inlineStr">
         <is>
-          <t>}</t>
+          <t>// ---- Toast feedback when filters change ----</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="24" t="inlineStr"/>
+      <c r="A58" s="24" t="inlineStr">
+        <is>
+          <t>function onEdit(e) {</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="24" t="inlineStr">
         <is>
-          <t>// ---- onEdit: live feedback when any filter changes ----</t>
+          <t xml:space="preserve">  const sheet = e.range.getSheet();</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="24" t="inlineStr">
         <is>
-          <t>function onEdit(e) {</t>
+          <t xml:space="preserve">  if (sheet.getName() !== 'Lookup') return;</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  const sheet = e.source.getActiveSheet();</t>
-        </is>
-      </c>
+      <c r="A61" s="24" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  if (sheet.getName() !== 'Lookup') return;</t>
+          <t xml:space="preserve">  const col  = e.range.getColumn();</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="24" t="inlineStr"/>
+      <c r="A63" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  const row  = e.range.getRow();</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  const col = e.range.getColumn();</t>
+          <t xml:space="preserve">  const ss   = e.source;</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  const row = e.range.getRow();</t>
-        </is>
-      </c>
+      <c r="A65" s="24" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  const ss  = e.source;</t>
+          <t xml:space="preserve">  // State cells (C or E, rows 6-51) updated by onSelectionChange</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="24" t="inlineStr"/>
+      <c r="A67" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  if ((col === 3 || col === 5) &amp;&amp; row &gt;= 6 &amp;&amp; row &lt;= 51) {</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  // County checkbox columns C (3) or E (5), rows 6-51</t>
+          <t xml:space="preserve">    const n = sheet.getRange('C6:C51').getValues().flat().filter(Boolean).length</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  if ((col === 3 || col === 5) &amp;&amp; row &gt;= 6 &amp;&amp; row &lt;= 51) {</t>
+          <t xml:space="preserve">            + sheet.getRange('E6:E51').getValues().flat().filter(Boolean).length;</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    const n = sheet.getRange('C6:C51').getValues().flat().filter(Boolean).length</t>
+          <t xml:space="preserve">    ss.toast(</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">            + sheet.getRange('E6:E51').getValues().flat().filter(Boolean).length;</t>
+          <t xml:space="preserve">      n === 0 ? 'All 92 counties shown.' : n + ' ' + (n === 1 ? 'county' : 'counties') + ' selected.',</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ss.toast(</t>
+          <t xml:space="preserve">      'County Filter', 3</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">      n === 0 ? 'Showing all 92 counties.' : n + ' counties selected.',</t>
+          <t xml:space="preserve">    );</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">      'County Filter', 3</t>
+          <t xml:space="preserve">    return;</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    );</t>
+          <t xml:space="preserve">  }</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    return;</t>
-        </is>
-      </c>
+      <c r="A76" s="24" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  }</t>
+          <t xml:space="preserve">  // District type dropdown (I4) or district number input (L4)</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="24" t="inlineStr"/>
+      <c r="A78" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  const addr = e.range.getA1Notation();</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  // District Type dropdown (I4) or District # input (L4)</t>
+          <t xml:space="preserve">  if (addr === 'I4' || addr === 'L4') {</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  const addr = e.range.getA1Notation();</t>
+          <t xml:space="preserve">    const type = sheet.getRange('I4').getValue() || 'All Types';</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  if (addr === 'I4' || addr === 'L4') {</t>
+          <t xml:space="preserve">    const num  = sheet.getRange('L4').getValue();</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    const type = sheet.getRange('I4').getValue();</t>
+          <t xml:space="preserve">    ss.toast(</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    const num  = sheet.getRange('L4').getValue();</t>
+          <t xml:space="preserve">      'Showing: ' + type + (num ? ', District ' + num : ', all districts'),</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ss.toast(</t>
+          <t xml:space="preserve">      'District Filter', 3</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">      'Filter: ' + (type || 'All Types') + (num ? ', District ' + num : ''),</t>
+          <t xml:space="preserve">    );</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">      'District Filter', 3</t>
+          <t xml:space="preserve">  }</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    );</t>
+          <t>}</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  }</t>
-        </is>
-      </c>
+      <c r="A88" s="24" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="24" t="inlineStr">
         <is>
-          <t>}</t>
+          <t>// ---- Bulk county helpers ----</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="24" t="inlineStr"/>
+      <c r="A90" s="24" t="inlineStr">
+        <is>
+          <t>function selectAllCounties() {</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="24" t="inlineStr">
         <is>
-          <t>function goToByDistrict() {</t>
+          <t xml:space="preserve">  const lu = SpreadsheetApp.getActiveSpreadsheet().getSheetByName('Lookup');</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  const ss = SpreadsheetApp.getActiveSpreadsheet();</t>
+          <t xml:space="preserve">  lu.getRange('C6:C51').setValue(true);</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ss.setActiveSheet(ss.getSheetByName('By District'));</t>
+          <t xml:space="preserve">  lu.getRange('E6:E51').setValue(true);</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SpreadsheetApp.getActiveSpreadsheet().toast('All 92 counties selected.', 'IRS Tools', 3);</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="24" t="inlineStr">
+        <is>
+          <t>}</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="24" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="24" t="inlineStr">
+        <is>
+          <t>function clearAllCounties() {</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  const lu = SpreadsheetApp.getActiveSpreadsheet().getSheetByName('Lookup');</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  lu.getRange('C6:C51').setValue(false);</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  lu.getRange('E6:E51').setValue(false);</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SpreadsheetApp.getActiveSpreadsheet().toast('Showing all 92 counties.', 'IRS Tools', 3);</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="24" t="inlineStr">
+        <is>
+          <t>}</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="24" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="24" t="inlineStr">
+        <is>
+          <t>// ---- Reset district filter ----</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="24" t="inlineStr">
+        <is>
+          <t>function resetDistrictFilter() {</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  const lu = SpreadsheetApp.getActiveSpreadsheet().getSheetByName('Lookup');</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  lu.getRange('I4').setValue('All Types');</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  lu.getRange('L4').clearContent();</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SpreadsheetApp.getActiveSpreadsheet().toast('District filter cleared.', 'IRS Tools', 2);</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="24" t="inlineStr">
+        <is>
+          <t>}</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="24" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="24" t="inlineStr">
+        <is>
+          <t>function goToByDistrict() {</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  const ss = SpreadsheetApp.getActiveSpreadsheet();</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ss.setActiveSheet(ss.getSheetByName('By District'));</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="24" t="inlineStr">
         <is>
           <t>}</t>
         </is>

</xml_diff>